<commit_message>
feat(sim): complete 1-iteration benchmark across 32 conditions and export master Excel workbook
</commit_message>
<xml_diff>
--- a/sim/simulation_experiments_grid.xlsx
+++ b/sim/simulation_experiments_grid.xlsx
@@ -1886,7 +1886,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H40"/>
+  <dimension ref="A1:H42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2448,7 +2448,7 @@
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>Proportion of days covered: (1/tau) * sum_{t=1}^tau I(band_lower(t) &lt;= RD_true(t) &lt;= band_upper(t)).</t>
+          <t>Proportion of days covered: (1/tau) * sum_{t=1}^tau I(band_lower(t) &lt;= RD_true(t) &lt;= band_upper(t)). Evaluated for TMLE and CCW-KM.</t>
         </is>
       </c>
       <c r="E24" s="14" t="n"/>
@@ -2478,7 +2478,7 @@
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>Average band width: (1/tau) * sum_{t=1}^tau [band_upper(t) - band_lower(t)].</t>
+          <t>Average band width: (1/tau) * sum_{t=1}^tau [band_upper(t) - band_lower(t)]. Evaluated for TMLE and CCW-KM.</t>
         </is>
       </c>
       <c r="E25" s="14" t="n"/>
@@ -2490,91 +2490,91 @@
       <c r="G25" s="14" t="n"/>
       <c r="H25" s="14" t="n"/>
     </row>
-    <row r="27" ht="24" customHeight="1">
-      <c r="A27" s="8" t="inlineStr">
+    <row r="26" ht="26" customHeight="1">
+      <c r="A26" s="13" t="inlineStr">
+        <is>
+          <t>elapsed_sec</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>Scalar</t>
+        </is>
+      </c>
+      <c r="C26" s="4" t="inlineStr">
+        <is>
+          <t>Numeric (sec)</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>Wall-clock elapsed execution time in seconds: proc.time()['elapsed'] - t_start.</t>
+        </is>
+      </c>
+      <c r="E26" s="14" t="n"/>
+      <c r="F26" s="5" t="inlineStr">
+        <is>
+          <t>Computational scalability and runtime benchmarking.</t>
+        </is>
+      </c>
+      <c r="G26" s="14" t="n"/>
+      <c r="H26" s="14" t="n"/>
+    </row>
+    <row r="28" ht="24" customHeight="1">
+      <c r="A28" s="8" t="inlineStr">
         <is>
           <t>3. ACROSS-RUN MONTE CARLO EVALUATION METRICS (AGGREGATED ACROSS B = 1,000 ITERATIONS)</t>
         </is>
       </c>
     </row>
-    <row r="28" ht="24" customHeight="1">
-      <c r="A28" s="9" t="inlineStr">
+    <row r="29" ht="24" customHeight="1">
+      <c r="A29" s="9" t="inlineStr">
         <is>
           <t>Metric Name</t>
         </is>
       </c>
-      <c r="B28" s="9" t="inlineStr">
+      <c r="B29" s="9" t="inlineStr">
         <is>
           <t>Mathematical Formula</t>
         </is>
       </c>
-      <c r="C28" s="9" t="inlineStr">
+      <c r="C29" s="9" t="inlineStr">
         <is>
           <t>Target / Optimal Value</t>
         </is>
       </c>
-      <c r="D28" s="9" t="inlineStr">
+      <c r="D29" s="9" t="inlineStr">
         <is>
           <t>Interpretation &amp; Significance</t>
         </is>
       </c>
-      <c r="E28" s="11" t="n"/>
-    </row>
-    <row r="29" ht="28" customHeight="1">
-      <c r="A29" s="12" t="inlineStr">
-        <is>
-          <t>Monte Carlo Mean</t>
-        </is>
-      </c>
-      <c r="B29" s="13" t="inlineStr">
-        <is>
-          <t>theta_bar = (1/B) sum_{b=1}^B psi_hat^(b)</t>
-        </is>
-      </c>
-      <c r="C29" s="15" t="inlineStr">
-        <is>
-          <t>theta_true</t>
-        </is>
-      </c>
-      <c r="D29" s="5" t="inlineStr">
-        <is>
-          <t>Average point estimate across all simulation iterations.</t>
-        </is>
-      </c>
-      <c r="E29" s="14" t="n"/>
-      <c r="F29" s="4" t="inlineStr">
-        <is>
-          <t>Estimator Performance</t>
-        </is>
-      </c>
-      <c r="G29" s="14" t="n"/>
-      <c r="H29" s="14" t="n"/>
+      <c r="E29" s="11" t="n"/>
     </row>
     <row r="30" ht="28" customHeight="1">
       <c r="A30" s="12" t="inlineStr">
         <is>
-          <t>Absolute Bias</t>
+          <t>Monte Carlo Mean</t>
         </is>
       </c>
       <c r="B30" s="13" t="inlineStr">
         <is>
-          <t>Bias = theta_bar - theta_true</t>
+          <t>theta_bar = (1/B) sum_{b=1}^B psi_hat^(b)</t>
         </is>
       </c>
       <c r="C30" s="15" t="inlineStr">
         <is>
-          <t>0.000</t>
+          <t>theta_true</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
         <is>
-          <t>Systematic deviation from true population parameter. Unbiasedness requires Bias -&gt; 0.</t>
+          <t>Average point estimate across all simulation iterations.</t>
         </is>
       </c>
       <c r="E30" s="14" t="n"/>
       <c r="F30" s="4" t="inlineStr">
         <is>
-          <t>Accuracy</t>
+          <t>Estimator Performance</t>
         </is>
       </c>
       <c r="G30" s="14" t="n"/>
@@ -2583,22 +2583,22 @@
     <row r="31" ht="28" customHeight="1">
       <c r="A31" s="12" t="inlineStr">
         <is>
-          <t>Relative Bias (%)</t>
+          <t>Absolute Bias</t>
         </is>
       </c>
       <c r="B31" s="13" t="inlineStr">
         <is>
-          <t>RelBias = [(theta_bar - theta_true) / theta_true] * 100%</t>
+          <t>Bias = theta_bar - theta_true</t>
         </is>
       </c>
       <c r="C31" s="15" t="inlineStr">
         <is>
-          <t>0.0%</t>
+          <t>0.000</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>Standardized bias percentage relative to effect magnitude. |RelBias| &lt; 5% considered excellent.</t>
+          <t>Systematic deviation from true population parameter. Unbiasedness requires Bias -&gt; 0.</t>
         </is>
       </c>
       <c r="E31" s="14" t="n"/>
@@ -2613,28 +2613,28 @@
     <row r="32" ht="28" customHeight="1">
       <c r="A32" s="12" t="inlineStr">
         <is>
-          <t>Empirical Standard Error (EmpSE)</t>
+          <t>Relative Bias (%)</t>
         </is>
       </c>
       <c r="B32" s="13" t="inlineStr">
         <is>
-          <t>EmpSE = sqrt( (1/(B-1)) sum_{b=1}^B (psi_hat^(b) - theta_bar)^2 )</t>
+          <t>RelBias = [(theta_bar - theta_true) / theta_true] * 100%</t>
         </is>
       </c>
       <c r="C32" s="15" t="inlineStr">
         <is>
-          <t>Minimal (Cramer-Rao / EIC Bound)</t>
+          <t>0.0%</t>
         </is>
       </c>
       <c r="D32" s="5" t="inlineStr">
         <is>
-          <t>True sampling variability of the estimator across repeated datasets. Gold standard variance benchmark.</t>
+          <t>Standardized bias percentage relative to effect magnitude. |RelBias| &lt; 5% considered excellent.</t>
         </is>
       </c>
       <c r="E32" s="14" t="n"/>
       <c r="F32" s="4" t="inlineStr">
         <is>
-          <t>Efficiency</t>
+          <t>Accuracy</t>
         </is>
       </c>
       <c r="G32" s="14" t="n"/>
@@ -2643,51 +2643,51 @@
     <row r="33" ht="28" customHeight="1">
       <c r="A33" s="12" t="inlineStr">
         <is>
+          <t>Empirical Standard Error (EmpSE)</t>
+        </is>
+      </c>
+      <c r="B33" s="13" t="inlineStr">
+        <is>
+          <t>EmpSE = sqrt( (1/(B-1)) sum_{b=1}^B (psi_hat^(b) - theta_bar)^2 )</t>
+        </is>
+      </c>
+      <c r="C33" s="15" t="inlineStr">
+        <is>
+          <t>Minimal (Cramer-Rao / EIC Bound)</t>
+        </is>
+      </c>
+      <c r="D33" s="5" t="inlineStr">
+        <is>
+          <t>True sampling variability of the estimator across repeated datasets. Gold standard variance benchmark.</t>
+        </is>
+      </c>
+      <c r="E33" s="14" t="n"/>
+      <c r="F33" s="4" t="inlineStr">
+        <is>
+          <t>Efficiency</t>
+        </is>
+      </c>
+      <c r="G33" s="14" t="n"/>
+      <c r="H33" s="14" t="n"/>
+    </row>
+    <row r="34" ht="28" customHeight="1">
+      <c r="A34" s="12" t="inlineStr">
+        <is>
           <t>Mean Model Standard Error (ModSE)</t>
         </is>
       </c>
-      <c r="B33" s="13" t="inlineStr">
+      <c r="B34" s="13" t="inlineStr">
         <is>
           <t>ModSE = (1/B) sum_{b=1}^B se_hat^(b)</t>
         </is>
       </c>
-      <c r="C33" s="15">
+      <c r="C34" s="15">
         <f> EmpSE</f>
         <v/>
       </c>
-      <c r="D33" s="5" t="inlineStr">
+      <c r="D34" s="5" t="inlineStr">
         <is>
           <t>Average standard error estimated internally by the model (via EIC or bootstrap).</t>
-        </is>
-      </c>
-      <c r="E33" s="14" t="n"/>
-      <c r="F33" s="4" t="inlineStr">
-        <is>
-          <t>Inference</t>
-        </is>
-      </c>
-      <c r="G33" s="14" t="n"/>
-      <c r="H33" s="14" t="n"/>
-    </row>
-    <row r="34" ht="28" customHeight="1">
-      <c r="A34" s="12" t="inlineStr">
-        <is>
-          <t>Standard Error Ratio</t>
-        </is>
-      </c>
-      <c r="B34" s="13" t="inlineStr">
-        <is>
-          <t>SE_Ratio = ModSE / EmpSE</t>
-        </is>
-      </c>
-      <c r="C34" s="15" t="inlineStr">
-        <is>
-          <t>1.000 (Range: 0.95 - 1.05)</t>
-        </is>
-      </c>
-      <c r="D34" s="5" t="inlineStr">
-        <is>
-          <t>Measures validity of variance estimator. &lt; 0.95 indicates anti-conservative inference; &gt; 1.05 indicates over-conservative.</t>
         </is>
       </c>
       <c r="E34" s="14" t="n"/>
@@ -2702,28 +2702,28 @@
     <row r="35" ht="28" customHeight="1">
       <c r="A35" s="12" t="inlineStr">
         <is>
-          <t>Pointwise 95% Coverage</t>
+          <t>Standard Error Ratio</t>
         </is>
       </c>
       <c r="B35" s="13" t="inlineStr">
         <is>
-          <t>Cov95(t) = (1/B) sum_{b=1}^B I( CI_L^(b)(t) &lt;= theta_true(t) &lt;= CI_U^(b)(t) )</t>
+          <t>SE_Ratio = ModSE / EmpSE</t>
         </is>
       </c>
       <c r="C35" s="15" t="inlineStr">
         <is>
-          <t>0.950 (95.0%)</t>
+          <t>1.000 (Range: 0.95 - 1.05)</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>Empirical coverage of pointwise confidence intervals at t=15 and t=30. Minimum acceptable: 93.5% for B=1000.</t>
+          <t>Measures validity of variance estimator. &lt; 0.95 indicates anti-conservative inference; &gt; 1.05 indicates over-conservative.</t>
         </is>
       </c>
       <c r="E35" s="14" t="n"/>
       <c r="F35" s="4" t="inlineStr">
         <is>
-          <t>Coverage</t>
+          <t>Inference</t>
         </is>
       </c>
       <c r="G35" s="14" t="n"/>
@@ -2732,28 +2732,28 @@
     <row r="36" ht="28" customHeight="1">
       <c r="A36" s="12" t="inlineStr">
         <is>
-          <t>Uniform Simultaneous Band Coverage</t>
+          <t>Pointwise 95% Coverage</t>
         </is>
       </c>
       <c r="B36" s="13" t="inlineStr">
         <is>
-          <t>Cov_simul = (1/B) sum_{b=1}^B I( forall t: band_L^(b)(t) &lt;= RD_true(t) &lt;= band_U^(b)(t) )</t>
+          <t>Cov95(t) = (1/B) sum_{b=1}^B I( CI_L^(b)(t) &lt;= theta_true(t) &lt;= CI_U^(b)(t) )</t>
         </is>
       </c>
       <c r="C36" s="15" t="inlineStr">
         <is>
-          <t>&gt;= 0.950 (95.0%)</t>
+          <t>0.950 (95.0%)</t>
         </is>
       </c>
       <c r="D36" s="5" t="inlineStr">
         <is>
-          <t>Strict simultaneous coverage: proportion of iterations where entire curve is covered over all 30 days.</t>
+          <t>Empirical coverage of pointwise confidence intervals at t=15 and t=30. Minimum acceptable: 93.5% for B=1000.</t>
         </is>
       </c>
       <c r="E36" s="14" t="n"/>
       <c r="F36" s="4" t="inlineStr">
         <is>
-          <t>Simultaneous Inference</t>
+          <t>Coverage</t>
         </is>
       </c>
       <c r="G36" s="14" t="n"/>
@@ -2762,28 +2762,28 @@
     <row r="37" ht="28" customHeight="1">
       <c r="A37" s="12" t="inlineStr">
         <is>
-          <t>Mean Pointwise Band Coverage (P_band)</t>
+          <t>Uniform Simultaneous Band Coverage</t>
         </is>
       </c>
       <c r="B37" s="13" t="inlineStr">
         <is>
-          <t>P_band_bar = (1/B) sum_{b=1}^B P_band^(b)</t>
+          <t>Cov_simul = (1/B) sum_{b=1}^B I( forall t: band_L^(b)(t) &lt;= RD_true(t) &lt;= band_U^(b)(t) )</t>
         </is>
       </c>
       <c r="C37" s="15" t="inlineStr">
         <is>
-          <t>&gt;= 0.980 (98.0%)</t>
+          <t>&gt;= 0.950 (95.0%)</t>
         </is>
       </c>
       <c r="D37" s="5" t="inlineStr">
         <is>
-          <t>Average percentage of the 30-day timeline bounded by the simultaneous band. Quantifies trajectory robustness.</t>
+          <t>Strict simultaneous coverage: proportion of iterations where entire curve is covered over all 30 days.</t>
         </is>
       </c>
       <c r="E37" s="14" t="n"/>
       <c r="F37" s="4" t="inlineStr">
         <is>
-          <t>Banded Trajectory</t>
+          <t>Simultaneous Inference</t>
         </is>
       </c>
       <c r="G37" s="14" t="n"/>
@@ -2792,28 +2792,28 @@
     <row r="38" ht="28" customHeight="1">
       <c r="A38" s="12" t="inlineStr">
         <is>
-          <t>Mean Band Width</t>
+          <t>Mean Pointwise Band Coverage (P_band)</t>
         </is>
       </c>
       <c r="B38" s="13" t="inlineStr">
         <is>
-          <t>Width_bar = (1/(B*tau)) sum_{b=1}^B sum_{t=1}^tau [band_U^(b)(t) - band_L^(b)(t)]</t>
+          <t>P_band_bar = (1/B) sum_{b=1}^B P_band^(b)</t>
         </is>
       </c>
       <c r="C38" s="15" t="inlineStr">
         <is>
-          <t>Minimal subject to Cov &gt;= 95%</t>
+          <t>&gt;= 0.980 (98.0%)</t>
         </is>
       </c>
       <c r="D38" s="5" t="inlineStr">
         <is>
-          <t>Quantifies precision of simultaneous bands. Tighter bands indicate superior statistical efficiency.</t>
+          <t>Average percentage of the 30-day timeline bounded by the simultaneous band. Quantifies trajectory robustness.</t>
         </is>
       </c>
       <c r="E38" s="14" t="n"/>
       <c r="F38" s="4" t="inlineStr">
         <is>
-          <t>Efficiency</t>
+          <t>Banded Trajectory</t>
         </is>
       </c>
       <c r="G38" s="14" t="n"/>
@@ -2822,28 +2822,28 @@
     <row r="39" ht="28" customHeight="1">
       <c r="A39" s="12" t="inlineStr">
         <is>
-          <t>Statistical Power (1 - beta)</t>
+          <t>Mean Band Width</t>
         </is>
       </c>
       <c r="B39" s="13" t="inlineStr">
         <is>
-          <t>Power = (1/B) sum_{b=1}^B I( p_val_30^(b) &lt; 0.05 )</t>
+          <t>Width_bar = (1/(B*tau)) sum_{b=1}^B sum_{t=1}^tau [band_U^(b)(t) - band_L^(b)(t)]</t>
         </is>
       </c>
       <c r="C39" s="15" t="inlineStr">
         <is>
-          <t>1.000 (100.0%)</t>
+          <t>Minimal subject to Cov &gt;= 95%</t>
         </is>
       </c>
       <c r="D39" s="5" t="inlineStr">
         <is>
-          <t>Probability of correctly rejecting null H0: RD(30)=0 given true benefit exists. Driven by efficiency.</t>
+          <t>Quantifies precision of simultaneous bands. Tighter bands indicate superior statistical efficiency.</t>
         </is>
       </c>
       <c r="E39" s="14" t="n"/>
       <c r="F39" s="4" t="inlineStr">
         <is>
-          <t>Hypothesis Testing</t>
+          <t>Efficiency</t>
         </is>
       </c>
       <c r="G39" s="14" t="n"/>
@@ -2852,22 +2852,22 @@
     <row r="40" ht="28" customHeight="1">
       <c r="A40" s="12" t="inlineStr">
         <is>
-          <t>False Negative Rate (beta / FNR)</t>
+          <t>Statistical Power (1 - beta)</t>
         </is>
       </c>
       <c r="B40" s="13" t="inlineStr">
         <is>
-          <t>FNR = 1.0 - Power</t>
+          <t>Power = (1/B) sum_{b=1}^B I( p_val_30^(b) &lt; 0.05 )</t>
         </is>
       </c>
       <c r="C40" s="15" t="inlineStr">
         <is>
-          <t>0.000 (0.0%)</t>
+          <t>1.000 (100.0%)</t>
         </is>
       </c>
       <c r="D40" s="5" t="inlineStr">
         <is>
-          <t>Probability of falsely concluding no treatment benefit exists (Type II error). Exposes cost of inefficient models.</t>
+          <t>Probability of correctly rejecting null H0: RD(30)=0 given true benefit exists. Driven by efficiency.</t>
         </is>
       </c>
       <c r="E40" s="14" t="n"/>
@@ -2879,8 +2879,68 @@
       <c r="G40" s="14" t="n"/>
       <c r="H40" s="14" t="n"/>
     </row>
+    <row r="41" ht="28" customHeight="1">
+      <c r="A41" s="12" t="inlineStr">
+        <is>
+          <t>False Negative Rate (beta / FNR)</t>
+        </is>
+      </c>
+      <c r="B41" s="13" t="inlineStr">
+        <is>
+          <t>FNR = 1.0 - Power</t>
+        </is>
+      </c>
+      <c r="C41" s="15" t="inlineStr">
+        <is>
+          <t>0.000 (0.0%)</t>
+        </is>
+      </c>
+      <c r="D41" s="5" t="inlineStr">
+        <is>
+          <t>Probability of falsely concluding no treatment benefit exists (Type II error). Exposes cost of inefficient models.</t>
+        </is>
+      </c>
+      <c r="E41" s="14" t="n"/>
+      <c r="F41" s="4" t="inlineStr">
+        <is>
+          <t>Hypothesis Testing</t>
+        </is>
+      </c>
+      <c r="G41" s="14" t="n"/>
+      <c r="H41" s="14" t="n"/>
+    </row>
+    <row r="42" ht="28" customHeight="1">
+      <c r="A42" s="12" t="inlineStr">
+        <is>
+          <t>Mean Elapsed Runtime (sec)</t>
+        </is>
+      </c>
+      <c r="B42" s="13" t="inlineStr">
+        <is>
+          <t>Runtime_bar = (1/B) sum_{b=1}^B elapsed_sec^(b)</t>
+        </is>
+      </c>
+      <c r="C42" s="15" t="inlineStr">
+        <is>
+          <t>Minimal (seconds)</t>
+        </is>
+      </c>
+      <c r="D42" s="5" t="inlineStr">
+        <is>
+          <t>Computational speed, scaling profile across sample sizes, and practical feasibility.</t>
+        </is>
+      </c>
+      <c r="E42" s="14" t="n"/>
+      <c r="F42" s="4" t="inlineStr">
+        <is>
+          <t>Computational Benchmarking</t>
+        </is>
+      </c>
+      <c r="G42" s="14" t="n"/>
+      <c r="H42" s="14" t="n"/>
+    </row>
   </sheetData>
-  <mergeCells count="62">
+  <mergeCells count="66">
     <mergeCell ref="F20:H20"/>
     <mergeCell ref="D20:E20"/>
     <mergeCell ref="F21:H21"/>
@@ -2889,8 +2949,11 @@
     <mergeCell ref="F33:H33"/>
     <mergeCell ref="D19:E19"/>
     <mergeCell ref="D34:E34"/>
+    <mergeCell ref="F41:H41"/>
+    <mergeCell ref="F42:H42"/>
     <mergeCell ref="F32:H32"/>
     <mergeCell ref="F35:H35"/>
+    <mergeCell ref="F26:H26"/>
     <mergeCell ref="E7:H7"/>
     <mergeCell ref="A11:H11"/>
     <mergeCell ref="F17:H17"/>
@@ -2902,22 +2965,21 @@
     <mergeCell ref="F23:H23"/>
     <mergeCell ref="F38:H38"/>
     <mergeCell ref="F22:H22"/>
-    <mergeCell ref="F28:H28"/>
     <mergeCell ref="F13:H13"/>
     <mergeCell ref="F31:H31"/>
     <mergeCell ref="D13:E13"/>
     <mergeCell ref="D35:E35"/>
     <mergeCell ref="D32:E32"/>
+    <mergeCell ref="D26:E26"/>
+    <mergeCell ref="D41:E41"/>
     <mergeCell ref="D17:E17"/>
-    <mergeCell ref="A27:H27"/>
+    <mergeCell ref="F37:H37"/>
     <mergeCell ref="E5:H5"/>
-    <mergeCell ref="F37:H37"/>
     <mergeCell ref="F39:H39"/>
     <mergeCell ref="D16:E16"/>
     <mergeCell ref="E8:H8"/>
     <mergeCell ref="F14:H14"/>
     <mergeCell ref="D37:E37"/>
-    <mergeCell ref="D28:E28"/>
     <mergeCell ref="D18:E18"/>
     <mergeCell ref="F29:H29"/>
     <mergeCell ref="D12:E12"/>
@@ -2933,11 +2995,13 @@
     <mergeCell ref="D30:E30"/>
     <mergeCell ref="D15:E15"/>
     <mergeCell ref="D33:E33"/>
+    <mergeCell ref="D42:E42"/>
     <mergeCell ref="D29:E29"/>
     <mergeCell ref="E6:H6"/>
     <mergeCell ref="D23:E23"/>
+    <mergeCell ref="A28:H28"/>
+    <mergeCell ref="D14:E14"/>
     <mergeCell ref="D38:E38"/>
-    <mergeCell ref="D14:E14"/>
     <mergeCell ref="F40:H40"/>
     <mergeCell ref="F12:H12"/>
     <mergeCell ref="F30:H30"/>

</xml_diff>